<commit_message>
Revised input excel sheets, M1, M2, M3 bugs fixed.
</commit_message>
<xml_diff>
--- a/data_input/crop-specific_rule_maiz_sugar.xlsx
+++ b/data_input/crop-specific_rule_maiz_sugar.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pyaez_iiasa\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\pyaez_github_test_env\input\maize_sugarcane_reduction_tables\M2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0CB7D467-4F4E-4ABB-8B1F-5B5180FD15A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F552425D-C5A8-4C82-9E69-2B028D504232}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3915" yWindow="3585" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1980" yWindow="1350" windowWidth="26760" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -111,12 +111,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -131,12 +137,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -422,7 +432,7 @@
   <dimension ref="A1:F10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="5.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="11.5703125" customWidth="1"/>
@@ -451,155 +461,146 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
+      <c r="D2" s="2">
+        <v>0</v>
+      </c>
+      <c r="E2" s="2">
+        <v>0</v>
+      </c>
+      <c r="F2" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="A3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
+      <c r="D3" s="2">
+        <v>0</v>
+      </c>
+      <c r="E3" s="2">
+        <v>0</v>
+      </c>
+      <c r="F3" s="2">
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="A4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <f xml:space="preserve"> 0* 90</f>
         <v>0</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <f xml:space="preserve"> 0.167*90</f>
         <v>15.030000000000001</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <f xml:space="preserve"> 0.167*90</f>
         <v>15.030000000000001</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="A5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <f>0*365</f>
         <v>0</v>
       </c>
-      <c r="E5" s="1">
-        <f>0.167*365</f>
-        <v>60.955000000000005</v>
-      </c>
-      <c r="F5" s="1">
-        <f>0.167*365</f>
-        <v>60.955000000000005</v>
+      <c r="E5" s="3">
+        <v>61</v>
+      </c>
+      <c r="F5" s="3">
+        <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="A6" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="1">
-        <f>0.167*365</f>
-        <v>60.955000000000005</v>
-      </c>
-      <c r="E6" s="1">
-        <f>0.333*365</f>
-        <v>121.545</v>
-      </c>
-      <c r="F6" s="1">
-        <f>0.333*365</f>
-        <v>121.545</v>
+      <c r="D6" s="3">
+        <v>61</v>
+      </c>
+      <c r="E6" s="3">
+        <v>122</v>
+      </c>
+      <c r="F6" s="3">
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="A7" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="1">
-        <f>0.667*365</f>
-        <v>243.45500000000001</v>
-      </c>
-      <c r="E7" s="1">
-        <f>0.667*365</f>
-        <v>243.45500000000001</v>
-      </c>
-      <c r="F7" s="1">
-        <f>0.667*365</f>
-        <v>243.45500000000001</v>
+      <c r="D7" s="3">
+        <v>243</v>
+      </c>
+      <c r="E7" s="3">
+        <v>243</v>
+      </c>
+      <c r="F7" s="3">
+        <v>243</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="D8" s="1">
-        <f>0.083*365</f>
-        <v>30.295000000000002</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1">
+      <c r="D8" s="3">
+        <v>30</v>
+      </c>
+      <c r="E8" s="3">
+        <v>0</v>
+      </c>
+      <c r="F8" s="3">
         <v>0</v>
       </c>
     </row>
@@ -654,15 +655,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008864D41C708CC54AABC64DB9F8EC5160" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8280e7c680d5d724f4413038ca100d1d">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="aecedfd1-a701-4d39-be9b-da32a8dfc2a5" xmlns:ns3="6cc8ca2e-56d8-406d-8e41-68c6b727753a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a78283ead66d0e44d8e1b525c3947135" ns2:_="" ns3:_="">
     <xsd:import namespace="aecedfd1-a701-4d39-be9b-da32a8dfc2a5"/>
@@ -905,15 +897,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{479F62A5-0DB5-4AC7-AA2B-89AAFA4EBEA0}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33F6540B-C062-42AF-84FC-7EE9BBC15D62}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -930,4 +923,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{479F62A5-0DB5-4AC7-AA2B-89AAFA4EBEA0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>